<commit_message>
Vollmacht auf einer Seite, Ankreuzfelder automatisch, Bosch-Beileger
- Nachtext D kompakter (8,5 pt, Zeilen 5,2 mm) + Keep-together fuer
  Ort/Datum und beide Unterschriftszeilen: der Block wird notfalls ohne
  Auto-Umbruch in die Reserve vor der Fusszeile gezeichnet und steht nie
  allein auf einer letzten Seite (Referenz AN250096 Seite 11); Angebot 16
  jetzt 11 statt 12 Seiten, Dauertest mit langem Angebot
- Ankreuzfelder automatisch: Messstellenbetreiber bei iMSys (P02/016),
  Stromlieferant bei SpotDynamic (P03/017), Anmeldung/... immer;
  anhaenge.vollmacht_kreuze + Tests aller Varianten; docs Punkt 9
- Blatt Anhaenge der Logik v5: Bosch CS3800iAW.pdf bei WP-Paket
  Pos. 045-054 im Angebot (Datei liegt in anlagen/); neu eingelesen,
  Vorschau zeigt 5 Anhaenge bei P01+P03+Paket, Grenzfall 054 geprueft

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/konfigurator_logik_v5.xlsx
+++ b/konfigurator_logik_v5.xlsx
@@ -5330,7 +5330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -5426,15 +5426,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Bosch CS3800iAW.pdf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>wenn WP-Paket Pos. 045–054 im Angebot</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Angebotsbeileger zur angebotenen Wärmepumpe (Gerätebroschüre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>(weitere Zeilen ergänzen)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Regeln: 'immer' | 'wenn &lt;Frage&gt; = &lt;Antwort&gt;' | 'wenn Pos. &lt;Nr&gt; im Angebot'</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>PDFs in den Ordner anlagen/ legen</t>
         </is>

</xml_diff>

<commit_message>
Phase 50: Multi-Sparten-Erfassung (WP/PV/KL/WB)
- Sparten-Auswahl beim Erfassungsstart (Lead-Interessen vorausgewaehlt,
  weitere zuwaehlbar, bereits erfasste markiert, Entwuerfe fortsetzbar);
  je Sparte eine eigene Erfassung mit eigenem Protokoll
- Weiche je Sparte: WP aus Fragen, PV aus Fragen PV, KL aus Fragen KL
  (logik_fuer_sparte); WB startet immer direkt im Freitext
- Fragetyp Wiederholgruppe generisch: KO05 expandiert je Raum Klone
  KR01#1..n mit sauberer Reihenfolge, dynamische Optionsliste KR07 aus
  KO04, Darstellung je Raum in Seite, Ansicht und Protokoll-PDF
- PV/KL-Absenden -> immer individuell, direkt In TAIFUN zu schreiben
  (reine Erfassung); Sparten-Badge an Erfassung, Warteschlange und
  externem Angebotseintrag (konfigurator_typ = Sparte)
- Sparten-Filter in Erfassungs- und Angebotsliste; Statistik Je Sparte
- Webtest 22/22, Unit-Suite 82/82

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/konfigurator_logik_v5.xlsx
+++ b/konfigurator_logik_v5.xlsx
@@ -656,7 +656,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -679,13 +678,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -708,7 +705,6 @@
           <t>Freitext</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>immer</t>
@@ -741,13 +737,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -770,13 +764,11 @@
           <t>Freitext groß</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -809,7 +801,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -842,7 +833,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -875,7 +865,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -898,13 +887,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -937,7 +924,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -960,13 +946,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>nur wenn PD05 = Ja</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -999,7 +983,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1022,13 +1005,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1051,13 +1032,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1080,13 +1059,11 @@
           <t>Freitext groß</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1119,7 +1096,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1152,7 +1128,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1185,7 +1160,6 @@
           <t>nur wenn PA02 = Ja</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1218,7 +1192,6 @@
           <t>nur wenn PA02 = Nein</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1251,7 +1224,6 @@
           <t>nur wenn PA04 = Ja</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1284,7 +1256,6 @@
           <t>nur wenn PA04 = Ja</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1317,7 +1288,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1350,7 +1320,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1373,13 +1342,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1402,13 +1369,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1441,7 +1406,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1474,7 +1438,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1507,7 +1470,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1530,13 +1492,11 @@
           <t>Freitext groß</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1596,7 +1556,6 @@
           <t>Datum</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>immer</t>
@@ -1690,7 +1649,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1713,13 +1671,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>immer</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1752,7 +1708,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1785,7 +1740,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1808,7 +1762,6 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>immer</t>
@@ -1823,7 +1776,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Raum {n}</t>
+          <t>Räume</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1841,7 +1794,6 @@
           <t>Freitext</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>je Raum (KO05)</t>
@@ -1856,7 +1808,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Raum {n}</t>
+          <t>Räume</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1884,12 +1836,11 @@
           <t>je Raum (KO05)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Raum {n}</t>
+          <t>Räume</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1917,12 +1868,11 @@
           <t>je Raum (KO05)</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Raum {n}</t>
+          <t>Räume</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1950,12 +1900,11 @@
           <t>je Raum (KO05)</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raum {n}</t>
+          <t>Räume</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1983,12 +1932,11 @@
           <t>je Raum (KO05)</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Raum {n}</t>
+          <t>Räume</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2016,12 +1964,11 @@
           <t>je Raum (KO05)</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Raum {n}</t>
+          <t>Räume</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2086,7 +2033,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2119,7 +2065,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2152,7 +2097,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2185,7 +2129,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2218,7 +2161,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2251,7 +2193,6 @@
           <t>immer</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2311,7 +2252,6 @@
           <t>Datum</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>immer</t>
@@ -2647,13 +2587,11 @@
           <t>Freitext</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>nur wenn O06 = Nein</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2676,13 +2614,11 @@
           <t>Freitext</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>nur wenn O06 = Nein</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2705,13 +2641,11 @@
           <t>Freitext</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>nur wenn O06 = Nein</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -2899,7 +2833,6 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>nur wenn A14 = Ja</t>
@@ -3346,7 +3279,6 @@
           <t>nur wenn A08 = Stahl oder Kunststoff</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -3748,13 +3680,11 @@
           <t>Zahleneingabe</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>nur wenn H08 = Ja</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -4088,7 +4018,6 @@
           <t>nur wenn E02 = Nein</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4121,7 +4050,6 @@
           <t>nur wenn E04 = Ja</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -4432,7 +4360,6 @@
           <t>Datum</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>immer</t>
@@ -6258,7 +6185,6 @@
           <t>A15 folgt – Heizlast hat Vorrang vor der kWh-Zuordnung</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6276,7 +6202,6 @@
           <t>– (Paket weiter über A03/kWh)</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6294,7 +6219,6 @@
           <t>Leistungsklasse lt. Paketmatrix-Spalte „Heizlast“ merken (Vorrang vor A03)</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6312,7 +6236,6 @@
           <t>AMPEL: individuell – Grund: Leistungsklasse zu hoch</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6352,7 +6275,6 @@
           <t>–</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6370,7 +6292,6 @@
           <t>H09 folgt</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6388,7 +6309,6 @@
           <t>–</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6450,7 +6370,6 @@
           <t>–</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6490,7 +6409,6 @@
           <t>–</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6508,7 +6426,6 @@
           <t>Startwerte der Angebotsverfolgung – keine Artikel</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Bugfix: Pos. 065 kam bei WW-Speicher 300 l doppelt ins Angebot
- Ursache: Aktionszeile N03 = 300 l (+ Pos. 065 x1) UND Paketmatrix-
  Spalte WW 300 l lieferten den Artikel beide - die Mengen summierten
  sich im selben Block auf 2 Stueck
- Logik-Excel: Aktionszeile umgetextet auf AWE-Paket lt. Paketmatrix
  (inkl. Pos. 065) ohne eigene Artikel-Anweisung, Bemerkung ergaenzt
- Parser: Aktionszeilen mit lt. Paketmatrix tragen grundsaetzlich keine
  eigenen Artikel-Referenzen mehr - die Matrix ist die einzige Quelle,
  Positionsnummern im Text sind nur erlaeuternd
- Validierungswarnung Doppelte Artikelquelle: prueft ALLE Paketmatrix-
  Spalten gegen alle Aktionszeilen mit Artikeln (haette den Bug gemeldet)
- Tests: N02=Ja/N03=300 l -> genau 1x Pos. 065 (Menge 1), Aktionszeile
  ohne Artikel, keine Doppelquellen in den uebrigen Spalten, Waechter-
  Warnung bei kuenstlichem Duplikat; Suite 91/91, Abnahme 68/68

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/konfigurator_logik_v5.xlsx
+++ b/konfigurator_logik_v5.xlsx
@@ -5430,10 +5430,14 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>AWE-Paket lt. Paketmatrix + Pos. 065 ×1</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr"/>
+          <t>AWE-Paket lt. Paketmatrix (inkl. Pos. 065)</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Pos. 065 kommt AUSSCHLIESSLICH aus der Paketmatrix-Spalte WW 300 l – hier keine eigene Artikel-Anweisung</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">

</xml_diff>